<commit_message>
Remove duplicate enterprise context vendor IDs
</commit_message>
<xml_diff>
--- a/docs/enterprise-context/synthetic/apexretail/03-cmdb-applications-services.xlsx
+++ b/docs/enterprise-context/synthetic/apexretail/03-cmdb-applications-services.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1699" uniqueCount="357">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1699" uniqueCount="359">
   <si>
     <t>Dataset</t>
   </si>
@@ -670,6 +670,12 @@
   </si>
   <si>
     <t>Assortment Planning</t>
+  </si>
+  <si>
+    <t>VEN-RELEX</t>
+  </si>
+  <si>
+    <t>CON-RELEX-2026</t>
   </si>
   <si>
     <t>CI-SVC-011</t>
@@ -3656,10 +3662,10 @@
         <v>48</v>
       </c>
       <c r="K27" t="s">
-        <v>153</v>
+        <v>219</v>
       </c>
       <c r="L27" t="s">
-        <v>154</v>
+        <v>220</v>
       </c>
       <c r="M27" t="s">
         <v>94</v>
@@ -3691,16 +3697,16 @@
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B28" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C28" t="s">
         <v>112</v>
       </c>
       <c r="D28" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="E28" t="s">
         <v>88</v>
@@ -3736,7 +3742,7 @@
         <v>63</v>
       </c>
       <c r="P28" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="Q28" t="s">
         <v>95</v>
@@ -3756,16 +3762,16 @@
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B29" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C29" t="s">
         <v>120</v>
       </c>
       <c r="D29" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="E29" t="s">
         <v>89</v>
@@ -3786,10 +3792,10 @@
         <v>48</v>
       </c>
       <c r="K29" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="L29" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="M29" t="s">
         <v>196</v>
@@ -3801,7 +3807,7 @@
         <v>63</v>
       </c>
       <c r="P29" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="Q29" t="s">
         <v>95</v>
@@ -3821,16 +3827,16 @@
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B30" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="C30" t="s">
         <v>26</v>
       </c>
       <c r="D30" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="E30" t="s">
         <v>90</v>
@@ -3866,7 +3872,7 @@
         <v>63</v>
       </c>
       <c r="P30" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="Q30" t="s">
         <v>95</v>
@@ -3886,16 +3892,16 @@
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B31" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C31" t="s">
         <v>112</v>
       </c>
       <c r="D31" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="E31" t="s">
         <v>100</v>
@@ -3931,7 +3937,7 @@
         <v>63</v>
       </c>
       <c r="P31" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="Q31" t="s">
         <v>95</v>
@@ -3951,16 +3957,16 @@
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B32" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C32" t="s">
         <v>120</v>
       </c>
       <c r="D32" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="E32" t="s">
         <v>106</v>
@@ -3996,7 +4002,7 @@
         <v>63</v>
       </c>
       <c r="P32" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="Q32" t="s">
         <v>95</v>
@@ -4016,16 +4022,16 @@
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B33" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C33" t="s">
         <v>26</v>
       </c>
       <c r="D33" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E33" t="s">
         <v>114</v>
@@ -4061,7 +4067,7 @@
         <v>63</v>
       </c>
       <c r="P33" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="Q33" t="s">
         <v>95</v>
@@ -4081,10 +4087,10 @@
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B34" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C34" t="s">
         <v>112</v>
@@ -4126,7 +4132,7 @@
         <v>63</v>
       </c>
       <c r="P34" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="Q34" t="s">
         <v>95</v>
@@ -4146,10 +4152,10 @@
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B35" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C35" t="s">
         <v>120</v>
@@ -4176,10 +4182,10 @@
         <v>48</v>
       </c>
       <c r="K35" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="L35" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="M35" t="s">
         <v>94</v>
@@ -4191,7 +4197,7 @@
         <v>63</v>
       </c>
       <c r="P35" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="Q35" t="s">
         <v>95</v>
@@ -4211,10 +4217,10 @@
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B36" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C36" t="s">
         <v>26</v>
@@ -4241,10 +4247,10 @@
         <v>48</v>
       </c>
       <c r="K36" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="L36" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="M36" t="s">
         <v>196</v>
@@ -4256,7 +4262,7 @@
         <v>63</v>
       </c>
       <c r="P36" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="Q36" t="s">
         <v>95</v>
@@ -4276,10 +4282,10 @@
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B37" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C37" t="s">
         <v>112</v>
@@ -4306,10 +4312,10 @@
         <v>48</v>
       </c>
       <c r="K37" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="L37" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="M37" t="s">
         <v>196</v>
@@ -4321,7 +4327,7 @@
         <v>63</v>
       </c>
       <c r="P37" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="Q37" t="s">
         <v>95</v>
@@ -4341,10 +4347,10 @@
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B38" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C38" t="s">
         <v>120</v>
@@ -4371,10 +4377,10 @@
         <v>48</v>
       </c>
       <c r="K38" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="L38" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="M38" t="s">
         <v>57</v>
@@ -4386,7 +4392,7 @@
         <v>63</v>
       </c>
       <c r="P38" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="Q38" t="s">
         <v>95</v>
@@ -4406,10 +4412,10 @@
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B39" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="C39" t="s">
         <v>26</v>
@@ -4436,10 +4442,10 @@
         <v>48</v>
       </c>
       <c r="K39" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="L39" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="M39" t="s">
         <v>94</v>
@@ -4451,7 +4457,7 @@
         <v>63</v>
       </c>
       <c r="P39" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="Q39" t="s">
         <v>95</v>
@@ -4471,10 +4477,10 @@
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B40" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C40" t="s">
         <v>112</v>
@@ -4501,10 +4507,10 @@
         <v>48</v>
       </c>
       <c r="K40" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="L40" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="M40" t="s">
         <v>196</v>
@@ -4516,7 +4522,7 @@
         <v>63</v>
       </c>
       <c r="P40" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="Q40" t="s">
         <v>95</v>
@@ -4536,10 +4542,10 @@
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B41" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C41" t="s">
         <v>120</v>
@@ -4566,10 +4572,10 @@
         <v>48</v>
       </c>
       <c r="K41" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="L41" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="M41" t="s">
         <v>196</v>
@@ -4581,7 +4587,7 @@
         <v>63</v>
       </c>
       <c r="P41" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="Q41" t="s">
         <v>95</v>
@@ -4601,10 +4607,10 @@
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B42" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="C42" t="s">
         <v>26</v>
@@ -4631,10 +4637,10 @@
         <v>48</v>
       </c>
       <c r="K42" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="L42" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="M42" t="s">
         <v>57</v>
@@ -4646,7 +4652,7 @@
         <v>63</v>
       </c>
       <c r="P42" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="Q42" t="s">
         <v>95</v>
@@ -4666,10 +4672,10 @@
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B43" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="C43" t="s">
         <v>112</v>
@@ -4696,10 +4702,10 @@
         <v>48</v>
       </c>
       <c r="K43" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="L43" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="M43" t="s">
         <v>94</v>
@@ -4711,7 +4717,7 @@
         <v>63</v>
       </c>
       <c r="P43" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="Q43" t="s">
         <v>95</v>
@@ -4731,16 +4737,16 @@
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B44" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C44" t="s">
         <v>120</v>
       </c>
       <c r="D44" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="E44" t="s">
         <v>122</v>
@@ -4776,7 +4782,7 @@
         <v>63</v>
       </c>
       <c r="P44" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="Q44" t="s">
         <v>95</v>
@@ -4796,16 +4802,16 @@
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B45" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C45" t="s">
         <v>26</v>
       </c>
       <c r="D45" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="E45" t="s">
         <v>129</v>
@@ -4841,7 +4847,7 @@
         <v>63</v>
       </c>
       <c r="P45" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="Q45" t="s">
         <v>95</v>
@@ -4861,16 +4867,16 @@
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B46" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C46" t="s">
         <v>112</v>
       </c>
       <c r="D46" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="E46" t="s">
         <v>136</v>
@@ -4906,7 +4912,7 @@
         <v>63</v>
       </c>
       <c r="P46" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="Q46" t="s">
         <v>95</v>
@@ -4926,16 +4932,16 @@
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B47" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="C47" t="s">
         <v>120</v>
       </c>
       <c r="D47" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="E47" t="s">
         <v>142</v>
@@ -4971,7 +4977,7 @@
         <v>63</v>
       </c>
       <c r="P47" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="Q47" t="s">
         <v>95</v>
@@ -4991,16 +4997,16 @@
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B48" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="C48" t="s">
         <v>26</v>
       </c>
       <c r="D48" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="E48" t="s">
         <v>88</v>
@@ -5036,7 +5042,7 @@
         <v>63</v>
       </c>
       <c r="P48" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="Q48" t="s">
         <v>95</v>
@@ -5056,16 +5062,16 @@
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B49" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C49" t="s">
         <v>112</v>
       </c>
       <c r="D49" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E49" t="s">
         <v>89</v>
@@ -5101,7 +5107,7 @@
         <v>63</v>
       </c>
       <c r="P49" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="Q49" t="s">
         <v>95</v>
@@ -5121,10 +5127,10 @@
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B50" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C50" t="s">
         <v>120</v>
@@ -5166,7 +5172,7 @@
         <v>63</v>
       </c>
       <c r="P50" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="Q50" t="s">
         <v>95</v>
@@ -5186,10 +5192,10 @@
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B51" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C51" t="s">
         <v>26</v>
@@ -5231,7 +5237,7 @@
         <v>63</v>
       </c>
       <c r="P51" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="Q51" t="s">
         <v>95</v>
@@ -5251,10 +5257,10 @@
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B52" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="C52" t="s">
         <v>112</v>
@@ -5296,7 +5302,7 @@
         <v>63</v>
       </c>
       <c r="P52" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="Q52" t="s">
         <v>95</v>
@@ -5316,10 +5322,10 @@
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B53" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="C53" t="s">
         <v>120</v>
@@ -5361,7 +5367,7 @@
         <v>63</v>
       </c>
       <c r="P53" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="Q53" t="s">
         <v>95</v>
@@ -5381,10 +5387,10 @@
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B54" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="C54" t="s">
         <v>26</v>
@@ -5411,10 +5417,10 @@
         <v>48</v>
       </c>
       <c r="K54" t="s">
-        <v>153</v>
+        <v>219</v>
       </c>
       <c r="L54" t="s">
-        <v>154</v>
+        <v>220</v>
       </c>
       <c r="M54" t="s">
         <v>57</v>
@@ -5426,7 +5432,7 @@
         <v>63</v>
       </c>
       <c r="P54" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="Q54" t="s">
         <v>95</v>
@@ -5446,10 +5452,10 @@
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B55" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="C55" t="s">
         <v>112</v>
@@ -5491,7 +5497,7 @@
         <v>63</v>
       </c>
       <c r="P55" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="Q55" t="s">
         <v>95</v>
@@ -5511,10 +5517,10 @@
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B56" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="C56" t="s">
         <v>120</v>
@@ -5541,10 +5547,10 @@
         <v>48</v>
       </c>
       <c r="K56" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="L56" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="M56" t="s">
         <v>196</v>
@@ -5556,7 +5562,7 @@
         <v>63</v>
       </c>
       <c r="P56" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="Q56" t="s">
         <v>95</v>
@@ -5576,10 +5582,10 @@
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B57" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="C57" t="s">
         <v>26</v>
@@ -5621,7 +5627,7 @@
         <v>63</v>
       </c>
       <c r="P57" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="Q57" t="s">
         <v>95</v>
@@ -5641,10 +5647,10 @@
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B58" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="C58" t="s">
         <v>112</v>
@@ -5686,7 +5692,7 @@
         <v>63</v>
       </c>
       <c r="P58" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="Q58" t="s">
         <v>95</v>
@@ -5706,10 +5712,10 @@
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B59" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="C59" t="s">
         <v>120</v>
@@ -5751,7 +5757,7 @@
         <v>63</v>
       </c>
       <c r="P59" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="Q59" t="s">
         <v>95</v>
@@ -5771,16 +5777,16 @@
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B60" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="C60" t="s">
         <v>26</v>
       </c>
       <c r="D60" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="E60" t="s">
         <v>90</v>
@@ -5816,7 +5822,7 @@
         <v>63</v>
       </c>
       <c r="P60" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="Q60" t="s">
         <v>95</v>
@@ -5836,16 +5842,16 @@
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B61" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="C61" t="s">
         <v>112</v>
       </c>
       <c r="D61" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="E61" t="s">
         <v>100</v>
@@ -5881,7 +5887,7 @@
         <v>63</v>
       </c>
       <c r="P61" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="Q61" t="s">
         <v>95</v>
@@ -5901,16 +5907,16 @@
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B62" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="C62" t="s">
         <v>120</v>
       </c>
       <c r="D62" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="E62" t="s">
         <v>106</v>
@@ -5931,10 +5937,10 @@
         <v>48</v>
       </c>
       <c r="K62" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="L62" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="M62" t="s">
         <v>57</v>
@@ -5946,7 +5952,7 @@
         <v>63</v>
       </c>
       <c r="P62" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="Q62" t="s">
         <v>95</v>
@@ -5966,16 +5972,16 @@
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B63" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="C63" t="s">
         <v>26</v>
       </c>
       <c r="D63" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="E63" t="s">
         <v>114</v>
@@ -5996,10 +6002,10 @@
         <v>48</v>
       </c>
       <c r="K63" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="L63" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="M63" t="s">
         <v>94</v>
@@ -6011,7 +6017,7 @@
         <v>63</v>
       </c>
       <c r="P63" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="Q63" t="s">
         <v>95</v>
@@ -6031,16 +6037,16 @@
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B64" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="C64" t="s">
         <v>112</v>
       </c>
       <c r="D64" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="E64" t="s">
         <v>122</v>
@@ -6061,10 +6067,10 @@
         <v>48</v>
       </c>
       <c r="K64" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="L64" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="M64" t="s">
         <v>196</v>
@@ -6076,7 +6082,7 @@
         <v>63</v>
       </c>
       <c r="P64" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="Q64" t="s">
         <v>95</v>
@@ -6096,16 +6102,16 @@
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B65" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="C65" t="s">
         <v>120</v>
       </c>
       <c r="D65" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E65" t="s">
         <v>129</v>
@@ -6126,10 +6132,10 @@
         <v>48</v>
       </c>
       <c r="K65" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="L65" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="M65" t="s">
         <v>196</v>
@@ -6141,7 +6147,7 @@
         <v>63</v>
       </c>
       <c r="P65" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="Q65" t="s">
         <v>95</v>
@@ -6161,10 +6167,10 @@
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B66" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="C66" t="s">
         <v>26</v>
@@ -6191,10 +6197,10 @@
         <v>48</v>
       </c>
       <c r="K66" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="L66" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="M66" t="s">
         <v>57</v>
@@ -6206,7 +6212,7 @@
         <v>63</v>
       </c>
       <c r="P66" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="Q66" t="s">
         <v>95</v>
@@ -6226,10 +6232,10 @@
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B67" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="C67" t="s">
         <v>112</v>
@@ -6256,10 +6262,10 @@
         <v>48</v>
       </c>
       <c r="K67" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="L67" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="M67" t="s">
         <v>94</v>
@@ -6271,7 +6277,7 @@
         <v>63</v>
       </c>
       <c r="P67" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="Q67" t="s">
         <v>95</v>
@@ -6291,10 +6297,10 @@
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B68" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C68" t="s">
         <v>120</v>
@@ -6321,10 +6327,10 @@
         <v>48</v>
       </c>
       <c r="K68" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="L68" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="M68" t="s">
         <v>196</v>
@@ -6336,7 +6342,7 @@
         <v>63</v>
       </c>
       <c r="P68" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="Q68" t="s">
         <v>95</v>
@@ -6356,10 +6362,10 @@
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B69" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="C69" t="s">
         <v>26</v>
@@ -6386,10 +6392,10 @@
         <v>48</v>
       </c>
       <c r="K69" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="L69" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="M69" t="s">
         <v>196</v>
@@ -6401,7 +6407,7 @@
         <v>63</v>
       </c>
       <c r="P69" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="Q69" t="s">
         <v>95</v>
@@ -6421,10 +6427,10 @@
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B70" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="C70" t="s">
         <v>112</v>
@@ -6451,10 +6457,10 @@
         <v>48</v>
       </c>
       <c r="K70" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="L70" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="M70" t="s">
         <v>57</v>
@@ -6466,7 +6472,7 @@
         <v>63</v>
       </c>
       <c r="P70" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="Q70" t="s">
         <v>95</v>
@@ -6486,10 +6492,10 @@
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B71" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="C71" t="s">
         <v>120</v>
@@ -6531,7 +6537,7 @@
         <v>63</v>
       </c>
       <c r="P71" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="Q71" t="s">
         <v>95</v>
@@ -6551,10 +6557,10 @@
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B72" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="C72" t="s">
         <v>26</v>
@@ -6596,7 +6602,7 @@
         <v>63</v>
       </c>
       <c r="P72" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="Q72" t="s">
         <v>95</v>
@@ -6616,10 +6622,10 @@
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B73" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="C73" t="s">
         <v>112</v>
@@ -6661,7 +6667,7 @@
         <v>63</v>
       </c>
       <c r="P73" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="Q73" t="s">
         <v>95</v>
@@ -6681,10 +6687,10 @@
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B74" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="C74" t="s">
         <v>120</v>
@@ -6726,7 +6732,7 @@
         <v>63</v>
       </c>
       <c r="P74" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="Q74" t="s">
         <v>95</v>
@@ -6746,10 +6752,10 @@
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B75" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="C75" t="s">
         <v>26</v>
@@ -6791,7 +6797,7 @@
         <v>63</v>
       </c>
       <c r="P75" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="Q75" t="s">
         <v>95</v>
@@ -6811,16 +6817,16 @@
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B76" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="C76" t="s">
         <v>112</v>
       </c>
       <c r="D76" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="E76" t="s">
         <v>136</v>
@@ -6856,7 +6862,7 @@
         <v>63</v>
       </c>
       <c r="P76" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="Q76" t="s">
         <v>95</v>
@@ -6876,16 +6882,16 @@
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B77" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="C77" t="s">
         <v>120</v>
       </c>
       <c r="D77" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="E77" t="s">
         <v>142</v>
@@ -6921,7 +6927,7 @@
         <v>63</v>
       </c>
       <c r="P77" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="Q77" t="s">
         <v>95</v>
@@ -6941,16 +6947,16 @@
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B78" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C78" t="s">
         <v>26</v>
       </c>
       <c r="D78" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="E78" t="s">
         <v>88</v>
@@ -6986,7 +6992,7 @@
         <v>63</v>
       </c>
       <c r="P78" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="Q78" t="s">
         <v>95</v>
@@ -7006,16 +7012,16 @@
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B79" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="C79" t="s">
         <v>112</v>
       </c>
       <c r="D79" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="E79" t="s">
         <v>89</v>
@@ -7051,7 +7057,7 @@
         <v>63</v>
       </c>
       <c r="P79" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="Q79" t="s">
         <v>95</v>
@@ -7071,16 +7077,16 @@
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B80" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="C80" t="s">
         <v>120</v>
       </c>
       <c r="D80" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="E80" t="s">
         <v>90</v>
@@ -7116,7 +7122,7 @@
         <v>63</v>
       </c>
       <c r="P80" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="Q80" t="s">
         <v>95</v>
@@ -7136,16 +7142,16 @@
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B81" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="C81" t="s">
         <v>26</v>
       </c>
       <c r="D81" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E81" t="s">
         <v>100</v>
@@ -7166,10 +7172,10 @@
         <v>48</v>
       </c>
       <c r="K81" t="s">
-        <v>153</v>
+        <v>219</v>
       </c>
       <c r="L81" t="s">
-        <v>154</v>
+        <v>220</v>
       </c>
       <c r="M81" t="s">
         <v>196</v>
@@ -7181,7 +7187,7 @@
         <v>63</v>
       </c>
       <c r="P81" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="Q81" t="s">
         <v>95</v>
@@ -7201,10 +7207,10 @@
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B82" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="C82" t="s">
         <v>112</v>
@@ -7246,7 +7252,7 @@
         <v>63</v>
       </c>
       <c r="P82" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="Q82" t="s">
         <v>95</v>
@@ -7266,10 +7272,10 @@
     </row>
     <row r="83" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B83" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="C83" t="s">
         <v>120</v>
@@ -7296,10 +7302,10 @@
         <v>48</v>
       </c>
       <c r="K83" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="L83" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="M83" t="s">
         <v>94</v>
@@ -7311,7 +7317,7 @@
         <v>63</v>
       </c>
       <c r="P83" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="Q83" t="s">
         <v>95</v>

</xml_diff>

<commit_message>
Deduplicate client enterprise context vendor IDs
</commit_message>
<xml_diff>
--- a/docs/enterprise-context/synthetic/apexretail/03-cmdb-applications-services.xlsx
+++ b/docs/enterprise-context/synthetic/apexretail/03-cmdb-applications-services.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1699" uniqueCount="357">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1699" uniqueCount="359">
   <si>
     <t>Dataset</t>
   </si>
@@ -670,6 +670,12 @@
   </si>
   <si>
     <t>Assortment Planning</t>
+  </si>
+  <si>
+    <t>VEN-RELEX</t>
+  </si>
+  <si>
+    <t>CON-RELEX-2026</t>
   </si>
   <si>
     <t>CI-SVC-011</t>
@@ -3656,10 +3662,10 @@
         <v>48</v>
       </c>
       <c r="K27" t="s">
-        <v>153</v>
+        <v>219</v>
       </c>
       <c r="L27" t="s">
-        <v>154</v>
+        <v>220</v>
       </c>
       <c r="M27" t="s">
         <v>94</v>
@@ -3691,16 +3697,16 @@
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B28" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C28" t="s">
         <v>112</v>
       </c>
       <c r="D28" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="E28" t="s">
         <v>88</v>
@@ -3736,7 +3742,7 @@
         <v>63</v>
       </c>
       <c r="P28" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="Q28" t="s">
         <v>95</v>
@@ -3756,16 +3762,16 @@
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B29" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C29" t="s">
         <v>120</v>
       </c>
       <c r="D29" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="E29" t="s">
         <v>89</v>
@@ -3786,10 +3792,10 @@
         <v>48</v>
       </c>
       <c r="K29" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="L29" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="M29" t="s">
         <v>196</v>
@@ -3801,7 +3807,7 @@
         <v>63</v>
       </c>
       <c r="P29" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="Q29" t="s">
         <v>95</v>
@@ -3821,16 +3827,16 @@
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B30" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="C30" t="s">
         <v>26</v>
       </c>
       <c r="D30" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="E30" t="s">
         <v>90</v>
@@ -3866,7 +3872,7 @@
         <v>63</v>
       </c>
       <c r="P30" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="Q30" t="s">
         <v>95</v>
@@ -3886,16 +3892,16 @@
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B31" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C31" t="s">
         <v>112</v>
       </c>
       <c r="D31" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="E31" t="s">
         <v>100</v>
@@ -3931,7 +3937,7 @@
         <v>63</v>
       </c>
       <c r="P31" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="Q31" t="s">
         <v>95</v>
@@ -3951,16 +3957,16 @@
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B32" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C32" t="s">
         <v>120</v>
       </c>
       <c r="D32" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="E32" t="s">
         <v>106</v>
@@ -3996,7 +4002,7 @@
         <v>63</v>
       </c>
       <c r="P32" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="Q32" t="s">
         <v>95</v>
@@ -4016,16 +4022,16 @@
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B33" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C33" t="s">
         <v>26</v>
       </c>
       <c r="D33" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E33" t="s">
         <v>114</v>
@@ -4061,7 +4067,7 @@
         <v>63</v>
       </c>
       <c r="P33" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="Q33" t="s">
         <v>95</v>
@@ -4081,10 +4087,10 @@
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B34" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C34" t="s">
         <v>112</v>
@@ -4126,7 +4132,7 @@
         <v>63</v>
       </c>
       <c r="P34" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="Q34" t="s">
         <v>95</v>
@@ -4146,10 +4152,10 @@
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B35" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C35" t="s">
         <v>120</v>
@@ -4176,10 +4182,10 @@
         <v>48</v>
       </c>
       <c r="K35" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="L35" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="M35" t="s">
         <v>94</v>
@@ -4191,7 +4197,7 @@
         <v>63</v>
       </c>
       <c r="P35" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="Q35" t="s">
         <v>95</v>
@@ -4211,10 +4217,10 @@
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B36" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C36" t="s">
         <v>26</v>
@@ -4241,10 +4247,10 @@
         <v>48</v>
       </c>
       <c r="K36" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="L36" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="M36" t="s">
         <v>196</v>
@@ -4256,7 +4262,7 @@
         <v>63</v>
       </c>
       <c r="P36" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="Q36" t="s">
         <v>95</v>
@@ -4276,10 +4282,10 @@
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B37" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C37" t="s">
         <v>112</v>
@@ -4306,10 +4312,10 @@
         <v>48</v>
       </c>
       <c r="K37" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="L37" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="M37" t="s">
         <v>196</v>
@@ -4321,7 +4327,7 @@
         <v>63</v>
       </c>
       <c r="P37" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="Q37" t="s">
         <v>95</v>
@@ -4341,10 +4347,10 @@
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B38" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C38" t="s">
         <v>120</v>
@@ -4371,10 +4377,10 @@
         <v>48</v>
       </c>
       <c r="K38" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="L38" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="M38" t="s">
         <v>57</v>
@@ -4386,7 +4392,7 @@
         <v>63</v>
       </c>
       <c r="P38" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="Q38" t="s">
         <v>95</v>
@@ -4406,10 +4412,10 @@
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B39" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="C39" t="s">
         <v>26</v>
@@ -4436,10 +4442,10 @@
         <v>48</v>
       </c>
       <c r="K39" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="L39" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="M39" t="s">
         <v>94</v>
@@ -4451,7 +4457,7 @@
         <v>63</v>
       </c>
       <c r="P39" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="Q39" t="s">
         <v>95</v>
@@ -4471,10 +4477,10 @@
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B40" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C40" t="s">
         <v>112</v>
@@ -4501,10 +4507,10 @@
         <v>48</v>
       </c>
       <c r="K40" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="L40" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="M40" t="s">
         <v>196</v>
@@ -4516,7 +4522,7 @@
         <v>63</v>
       </c>
       <c r="P40" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="Q40" t="s">
         <v>95</v>
@@ -4536,10 +4542,10 @@
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B41" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C41" t="s">
         <v>120</v>
@@ -4566,10 +4572,10 @@
         <v>48</v>
       </c>
       <c r="K41" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="L41" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="M41" t="s">
         <v>196</v>
@@ -4581,7 +4587,7 @@
         <v>63</v>
       </c>
       <c r="P41" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="Q41" t="s">
         <v>95</v>
@@ -4601,10 +4607,10 @@
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B42" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="C42" t="s">
         <v>26</v>
@@ -4631,10 +4637,10 @@
         <v>48</v>
       </c>
       <c r="K42" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="L42" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="M42" t="s">
         <v>57</v>
@@ -4646,7 +4652,7 @@
         <v>63</v>
       </c>
       <c r="P42" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="Q42" t="s">
         <v>95</v>
@@ -4666,10 +4672,10 @@
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B43" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="C43" t="s">
         <v>112</v>
@@ -4696,10 +4702,10 @@
         <v>48</v>
       </c>
       <c r="K43" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="L43" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="M43" t="s">
         <v>94</v>
@@ -4711,7 +4717,7 @@
         <v>63</v>
       </c>
       <c r="P43" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="Q43" t="s">
         <v>95</v>
@@ -4731,16 +4737,16 @@
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B44" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C44" t="s">
         <v>120</v>
       </c>
       <c r="D44" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="E44" t="s">
         <v>122</v>
@@ -4776,7 +4782,7 @@
         <v>63</v>
       </c>
       <c r="P44" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="Q44" t="s">
         <v>95</v>
@@ -4796,16 +4802,16 @@
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B45" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C45" t="s">
         <v>26</v>
       </c>
       <c r="D45" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="E45" t="s">
         <v>129</v>
@@ -4841,7 +4847,7 @@
         <v>63</v>
       </c>
       <c r="P45" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="Q45" t="s">
         <v>95</v>
@@ -4861,16 +4867,16 @@
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B46" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C46" t="s">
         <v>112</v>
       </c>
       <c r="D46" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="E46" t="s">
         <v>136</v>
@@ -4906,7 +4912,7 @@
         <v>63</v>
       </c>
       <c r="P46" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="Q46" t="s">
         <v>95</v>
@@ -4926,16 +4932,16 @@
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B47" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="C47" t="s">
         <v>120</v>
       </c>
       <c r="D47" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="E47" t="s">
         <v>142</v>
@@ -4971,7 +4977,7 @@
         <v>63</v>
       </c>
       <c r="P47" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="Q47" t="s">
         <v>95</v>
@@ -4991,16 +4997,16 @@
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B48" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="C48" t="s">
         <v>26</v>
       </c>
       <c r="D48" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="E48" t="s">
         <v>88</v>
@@ -5036,7 +5042,7 @@
         <v>63</v>
       </c>
       <c r="P48" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="Q48" t="s">
         <v>95</v>
@@ -5056,16 +5062,16 @@
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B49" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C49" t="s">
         <v>112</v>
       </c>
       <c r="D49" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E49" t="s">
         <v>89</v>
@@ -5101,7 +5107,7 @@
         <v>63</v>
       </c>
       <c r="P49" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="Q49" t="s">
         <v>95</v>
@@ -5121,10 +5127,10 @@
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B50" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C50" t="s">
         <v>120</v>
@@ -5166,7 +5172,7 @@
         <v>63</v>
       </c>
       <c r="P50" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="Q50" t="s">
         <v>95</v>
@@ -5186,10 +5192,10 @@
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B51" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C51" t="s">
         <v>26</v>
@@ -5231,7 +5237,7 @@
         <v>63</v>
       </c>
       <c r="P51" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="Q51" t="s">
         <v>95</v>
@@ -5251,10 +5257,10 @@
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B52" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="C52" t="s">
         <v>112</v>
@@ -5296,7 +5302,7 @@
         <v>63</v>
       </c>
       <c r="P52" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="Q52" t="s">
         <v>95</v>
@@ -5316,10 +5322,10 @@
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B53" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="C53" t="s">
         <v>120</v>
@@ -5361,7 +5367,7 @@
         <v>63</v>
       </c>
       <c r="P53" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="Q53" t="s">
         <v>95</v>
@@ -5381,10 +5387,10 @@
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B54" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="C54" t="s">
         <v>26</v>
@@ -5411,10 +5417,10 @@
         <v>48</v>
       </c>
       <c r="K54" t="s">
-        <v>153</v>
+        <v>219</v>
       </c>
       <c r="L54" t="s">
-        <v>154</v>
+        <v>220</v>
       </c>
       <c r="M54" t="s">
         <v>57</v>
@@ -5426,7 +5432,7 @@
         <v>63</v>
       </c>
       <c r="P54" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="Q54" t="s">
         <v>95</v>
@@ -5446,10 +5452,10 @@
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B55" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="C55" t="s">
         <v>112</v>
@@ -5491,7 +5497,7 @@
         <v>63</v>
       </c>
       <c r="P55" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="Q55" t="s">
         <v>95</v>
@@ -5511,10 +5517,10 @@
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B56" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="C56" t="s">
         <v>120</v>
@@ -5541,10 +5547,10 @@
         <v>48</v>
       </c>
       <c r="K56" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="L56" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="M56" t="s">
         <v>196</v>
@@ -5556,7 +5562,7 @@
         <v>63</v>
       </c>
       <c r="P56" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="Q56" t="s">
         <v>95</v>
@@ -5576,10 +5582,10 @@
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B57" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="C57" t="s">
         <v>26</v>
@@ -5621,7 +5627,7 @@
         <v>63</v>
       </c>
       <c r="P57" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="Q57" t="s">
         <v>95</v>
@@ -5641,10 +5647,10 @@
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B58" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="C58" t="s">
         <v>112</v>
@@ -5686,7 +5692,7 @@
         <v>63</v>
       </c>
       <c r="P58" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="Q58" t="s">
         <v>95</v>
@@ -5706,10 +5712,10 @@
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B59" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="C59" t="s">
         <v>120</v>
@@ -5751,7 +5757,7 @@
         <v>63</v>
       </c>
       <c r="P59" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="Q59" t="s">
         <v>95</v>
@@ -5771,16 +5777,16 @@
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B60" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="C60" t="s">
         <v>26</v>
       </c>
       <c r="D60" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="E60" t="s">
         <v>90</v>
@@ -5816,7 +5822,7 @@
         <v>63</v>
       </c>
       <c r="P60" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="Q60" t="s">
         <v>95</v>
@@ -5836,16 +5842,16 @@
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B61" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="C61" t="s">
         <v>112</v>
       </c>
       <c r="D61" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="E61" t="s">
         <v>100</v>
@@ -5881,7 +5887,7 @@
         <v>63</v>
       </c>
       <c r="P61" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="Q61" t="s">
         <v>95</v>
@@ -5901,16 +5907,16 @@
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B62" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="C62" t="s">
         <v>120</v>
       </c>
       <c r="D62" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="E62" t="s">
         <v>106</v>
@@ -5931,10 +5937,10 @@
         <v>48</v>
       </c>
       <c r="K62" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="L62" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="M62" t="s">
         <v>57</v>
@@ -5946,7 +5952,7 @@
         <v>63</v>
       </c>
       <c r="P62" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="Q62" t="s">
         <v>95</v>
@@ -5966,16 +5972,16 @@
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B63" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="C63" t="s">
         <v>26</v>
       </c>
       <c r="D63" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="E63" t="s">
         <v>114</v>
@@ -5996,10 +6002,10 @@
         <v>48</v>
       </c>
       <c r="K63" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="L63" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="M63" t="s">
         <v>94</v>
@@ -6011,7 +6017,7 @@
         <v>63</v>
       </c>
       <c r="P63" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="Q63" t="s">
         <v>95</v>
@@ -6031,16 +6037,16 @@
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B64" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="C64" t="s">
         <v>112</v>
       </c>
       <c r="D64" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="E64" t="s">
         <v>122</v>
@@ -6061,10 +6067,10 @@
         <v>48</v>
       </c>
       <c r="K64" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="L64" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="M64" t="s">
         <v>196</v>
@@ -6076,7 +6082,7 @@
         <v>63</v>
       </c>
       <c r="P64" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="Q64" t="s">
         <v>95</v>
@@ -6096,16 +6102,16 @@
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B65" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="C65" t="s">
         <v>120</v>
       </c>
       <c r="D65" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E65" t="s">
         <v>129</v>
@@ -6126,10 +6132,10 @@
         <v>48</v>
       </c>
       <c r="K65" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="L65" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="M65" t="s">
         <v>196</v>
@@ -6141,7 +6147,7 @@
         <v>63</v>
       </c>
       <c r="P65" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="Q65" t="s">
         <v>95</v>
@@ -6161,10 +6167,10 @@
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B66" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="C66" t="s">
         <v>26</v>
@@ -6191,10 +6197,10 @@
         <v>48</v>
       </c>
       <c r="K66" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="L66" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="M66" t="s">
         <v>57</v>
@@ -6206,7 +6212,7 @@
         <v>63</v>
       </c>
       <c r="P66" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="Q66" t="s">
         <v>95</v>
@@ -6226,10 +6232,10 @@
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B67" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="C67" t="s">
         <v>112</v>
@@ -6256,10 +6262,10 @@
         <v>48</v>
       </c>
       <c r="K67" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="L67" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="M67" t="s">
         <v>94</v>
@@ -6271,7 +6277,7 @@
         <v>63</v>
       </c>
       <c r="P67" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="Q67" t="s">
         <v>95</v>
@@ -6291,10 +6297,10 @@
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B68" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C68" t="s">
         <v>120</v>
@@ -6321,10 +6327,10 @@
         <v>48</v>
       </c>
       <c r="K68" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="L68" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="M68" t="s">
         <v>196</v>
@@ -6336,7 +6342,7 @@
         <v>63</v>
       </c>
       <c r="P68" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="Q68" t="s">
         <v>95</v>
@@ -6356,10 +6362,10 @@
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B69" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="C69" t="s">
         <v>26</v>
@@ -6386,10 +6392,10 @@
         <v>48</v>
       </c>
       <c r="K69" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="L69" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="M69" t="s">
         <v>196</v>
@@ -6401,7 +6407,7 @@
         <v>63</v>
       </c>
       <c r="P69" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="Q69" t="s">
         <v>95</v>
@@ -6421,10 +6427,10 @@
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B70" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="C70" t="s">
         <v>112</v>
@@ -6451,10 +6457,10 @@
         <v>48</v>
       </c>
       <c r="K70" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="L70" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="M70" t="s">
         <v>57</v>
@@ -6466,7 +6472,7 @@
         <v>63</v>
       </c>
       <c r="P70" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="Q70" t="s">
         <v>95</v>
@@ -6486,10 +6492,10 @@
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B71" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="C71" t="s">
         <v>120</v>
@@ -6531,7 +6537,7 @@
         <v>63</v>
       </c>
       <c r="P71" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="Q71" t="s">
         <v>95</v>
@@ -6551,10 +6557,10 @@
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B72" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="C72" t="s">
         <v>26</v>
@@ -6596,7 +6602,7 @@
         <v>63</v>
       </c>
       <c r="P72" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="Q72" t="s">
         <v>95</v>
@@ -6616,10 +6622,10 @@
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B73" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="C73" t="s">
         <v>112</v>
@@ -6661,7 +6667,7 @@
         <v>63</v>
       </c>
       <c r="P73" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="Q73" t="s">
         <v>95</v>
@@ -6681,10 +6687,10 @@
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B74" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="C74" t="s">
         <v>120</v>
@@ -6726,7 +6732,7 @@
         <v>63</v>
       </c>
       <c r="P74" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="Q74" t="s">
         <v>95</v>
@@ -6746,10 +6752,10 @@
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B75" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="C75" t="s">
         <v>26</v>
@@ -6791,7 +6797,7 @@
         <v>63</v>
       </c>
       <c r="P75" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="Q75" t="s">
         <v>95</v>
@@ -6811,16 +6817,16 @@
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B76" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="C76" t="s">
         <v>112</v>
       </c>
       <c r="D76" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="E76" t="s">
         <v>136</v>
@@ -6856,7 +6862,7 @@
         <v>63</v>
       </c>
       <c r="P76" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="Q76" t="s">
         <v>95</v>
@@ -6876,16 +6882,16 @@
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B77" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="C77" t="s">
         <v>120</v>
       </c>
       <c r="D77" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="E77" t="s">
         <v>142</v>
@@ -6921,7 +6927,7 @@
         <v>63</v>
       </c>
       <c r="P77" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="Q77" t="s">
         <v>95</v>
@@ -6941,16 +6947,16 @@
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B78" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C78" t="s">
         <v>26</v>
       </c>
       <c r="D78" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="E78" t="s">
         <v>88</v>
@@ -6986,7 +6992,7 @@
         <v>63</v>
       </c>
       <c r="P78" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="Q78" t="s">
         <v>95</v>
@@ -7006,16 +7012,16 @@
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B79" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="C79" t="s">
         <v>112</v>
       </c>
       <c r="D79" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="E79" t="s">
         <v>89</v>
@@ -7051,7 +7057,7 @@
         <v>63</v>
       </c>
       <c r="P79" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="Q79" t="s">
         <v>95</v>
@@ -7071,16 +7077,16 @@
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B80" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="C80" t="s">
         <v>120</v>
       </c>
       <c r="D80" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="E80" t="s">
         <v>90</v>
@@ -7116,7 +7122,7 @@
         <v>63</v>
       </c>
       <c r="P80" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="Q80" t="s">
         <v>95</v>
@@ -7136,16 +7142,16 @@
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B81" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="C81" t="s">
         <v>26</v>
       </c>
       <c r="D81" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E81" t="s">
         <v>100</v>
@@ -7166,10 +7172,10 @@
         <v>48</v>
       </c>
       <c r="K81" t="s">
-        <v>153</v>
+        <v>219</v>
       </c>
       <c r="L81" t="s">
-        <v>154</v>
+        <v>220</v>
       </c>
       <c r="M81" t="s">
         <v>196</v>
@@ -7181,7 +7187,7 @@
         <v>63</v>
       </c>
       <c r="P81" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="Q81" t="s">
         <v>95</v>
@@ -7201,10 +7207,10 @@
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B82" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="C82" t="s">
         <v>112</v>
@@ -7246,7 +7252,7 @@
         <v>63</v>
       </c>
       <c r="P82" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="Q82" t="s">
         <v>95</v>
@@ -7266,10 +7272,10 @@
     </row>
     <row r="83" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B83" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="C83" t="s">
         <v>120</v>
@@ -7296,10 +7302,10 @@
         <v>48</v>
       </c>
       <c r="K83" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="L83" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="M83" t="s">
         <v>94</v>
@@ -7311,7 +7317,7 @@
         <v>63</v>
       </c>
       <c r="P83" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="Q83" t="s">
         <v>95</v>

</xml_diff>